<commit_message>
📊 Full pipeline output Wed May  6 07:54:57 UTC 2026
</commit_message>
<xml_diff>
--- a/output/intraday/riepilogo_intraday_2026-05-06.xlsx
+++ b/output/intraday/riepilogo_intraday_2026-05-06.xlsx
@@ -802,7 +802,7 @@
         <v>46147</v>
       </c>
       <c r="C2" t="n">
-        <v>42.02</v>
+        <v>43.7</v>
       </c>
       <c r="D2" t="n">
         <v>3280000</v>
@@ -815,7 +815,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>-23.08%</t>
+          <t>-23.98%</t>
         </is>
       </c>
       <c r="H2" t="n">
@@ -1036,7 +1036,7 @@
         <v>46147</v>
       </c>
       <c r="C3" t="n">
-        <v>60.78</v>
+        <v>59.36</v>
       </c>
       <c r="D3" t="n">
         <v>13480000</v>
@@ -1049,7 +1049,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>-30.11%</t>
+          <t>-29.49%</t>
         </is>
       </c>
       <c r="H3" t="n">
@@ -1270,7 +1270,7 @@
         <v>46147</v>
       </c>
       <c r="C4" t="n">
-        <v>31.07</v>
+        <v>30.66</v>
       </c>
       <c r="D4" t="n">
         <v>842590000</v>
@@ -1283,7 +1283,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>24.39%</t>
+          <t>24.78%</t>
         </is>
       </c>
       <c r="H4" t="n">
@@ -1504,7 +1504,7 @@
         <v>46147</v>
       </c>
       <c r="C5" t="n">
-        <v>40.69</v>
+        <v>39.31</v>
       </c>
       <c r="D5" t="n">
         <v>2360000</v>
@@ -1517,7 +1517,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2.45%</t>
+          <t>3.47%</t>
         </is>
       </c>
       <c r="H5" t="n">

</xml_diff>